<commit_message>
low el prices case study setup
</commit_message>
<xml_diff>
--- a/data/carriers_data/naphtha_bio/naphtha_bio_availability.xlsx
+++ b/data/carriers_data/naphtha_bio/naphtha_bio_availability.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Github\AdOpT-NET0_my\data\carriers_data\naphtha_bio\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D6FD398-D18D-4667-B2E4-E0B1AE6847C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A157F25-E460-4EB7-A830-BA1E9E60FDCE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="768" yWindow="768" windowWidth="17280" windowHeight="8880" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="note" sheetId="2" r:id="rId1"/>

</xml_diff>